<commit_message>
TABLA STURGES: bien realizado
</commit_message>
<xml_diff>
--- a/OTROS/DATOS PRUEBA.xlsx
+++ b/OTROS/DATOS PRUEBA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Presi\Desktop\QUINTOSEMESTRE\Estadistica\R\AUTOAPRENDIZAJE-R\OTROS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5446FF-2CC6-4585-9463-6915EBF4608C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511F2A8A-B2DA-4CD3-96CF-736EC73B5D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="37">
   <si>
     <t>SIMPLE INSPECCION</t>
   </si>
@@ -85,6 +85,57 @@
   </si>
   <si>
     <t>STURGES</t>
+  </si>
+  <si>
+    <t>1.64</t>
+  </si>
+  <si>
+    <t>1.58</t>
+  </si>
+  <si>
+    <t>1.70</t>
+  </si>
+  <si>
+    <t>1.59</t>
+  </si>
+  <si>
+    <t>1.55</t>
+  </si>
+  <si>
+    <t>1.65</t>
+  </si>
+  <si>
+    <t>1.71</t>
+  </si>
+  <si>
+    <t>1.60</t>
+  </si>
+  <si>
+    <t>1.74</t>
+  </si>
+  <si>
+    <t>1.68</t>
+  </si>
+  <si>
+    <t>1.57</t>
+  </si>
+  <si>
+    <t>1.66</t>
+  </si>
+  <si>
+    <t>1.63</t>
+  </si>
+  <si>
+    <t>1.72</t>
+  </si>
+  <si>
+    <t>1.79</t>
+  </si>
+  <si>
+    <t>1.56</t>
+  </si>
+  <si>
+    <t>1.67</t>
   </si>
 </sst>
 </file>
@@ -405,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:K23"/>
+  <dimension ref="B1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.35">
@@ -852,6 +903,93 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" t="s">
+        <v>24</v>
+      </c>
+      <c r="G25" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" t="s">
+        <v>32</v>
+      </c>
+      <c r="I26" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" t="s">
+        <v>35</v>
+      </c>
+      <c r="J27" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B23:K23"/>

</xml_diff>

<commit_message>
EXCEL: mejorar datos prueba
</commit_message>
<xml_diff>
--- a/OTROS/DATOS PRUEBA.xlsx
+++ b/OTROS/DATOS PRUEBA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Presi\Desktop\QUINTOSEMESTRE\Estadistica\R\AUTOAPRENDIZAJE-R\OTROS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511F2A8A-B2DA-4CD3-96CF-736EC73B5D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF366EB3-5A0C-4456-98CF-951AC205E011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="54">
   <si>
     <t>SIMPLE INSPECCION</t>
   </si>
@@ -136,6 +136,57 @@
   </si>
   <si>
     <t>1.67</t>
+  </si>
+  <si>
+    <t>GRAFICO DE BARRAS</t>
+  </si>
+  <si>
+    <t>Pan</t>
+  </si>
+  <si>
+    <t>Leche</t>
+  </si>
+  <si>
+    <t>Arroz</t>
+  </si>
+  <si>
+    <t>Azúcar</t>
+  </si>
+  <si>
+    <t>Aceite</t>
+  </si>
+  <si>
+    <t>Fideo</t>
+  </si>
+  <si>
+    <t>DIAGRAMA LINEAL</t>
+  </si>
+  <si>
+    <t>Enero</t>
+  </si>
+  <si>
+    <t>Febrero</t>
+  </si>
+  <si>
+    <t>Marzo</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Septiembre</t>
   </si>
 </sst>
 </file>
@@ -456,10 +507,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:K27"/>
+  <dimension ref="B1:T27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="18" max="18" width="13.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,8 +526,34 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="M1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>120</v>
+      </c>
+      <c r="R3" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>7</v>
       </c>
@@ -504,8 +584,20 @@
       <c r="K4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="N4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4">
+        <v>85</v>
+      </c>
+      <c r="R4" t="s">
+        <v>46</v>
+      </c>
+      <c r="S4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>8</v>
       </c>
@@ -536,8 +628,20 @@
       <c r="K5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="N5" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5">
+        <v>64</v>
+      </c>
+      <c r="R5" t="s">
+        <v>47</v>
+      </c>
+      <c r="S5">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>9</v>
       </c>
@@ -568,8 +672,20 @@
       <c r="K6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="N6" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6">
+        <v>58</v>
+      </c>
+      <c r="R6" t="s">
+        <v>48</v>
+      </c>
+      <c r="S6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>11</v>
       </c>
@@ -600,8 +716,42 @@
       <c r="K7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="N7" t="s">
+        <v>42</v>
+      </c>
+      <c r="O7">
+        <v>42</v>
+      </c>
+      <c r="R7" t="s">
+        <v>49</v>
+      </c>
+      <c r="S7">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="N8" t="s">
+        <v>43</v>
+      </c>
+      <c r="O8">
+        <v>37</v>
+      </c>
+      <c r="R8" t="s">
+        <v>50</v>
+      </c>
+      <c r="S8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="R9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>13</v>
       </c>
@@ -632,8 +782,14 @@
       <c r="K10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="R10" t="s">
+        <v>52</v>
+      </c>
+      <c r="S10">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>17</v>
       </c>
@@ -664,8 +820,14 @@
       <c r="K11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="R11" t="s">
+        <v>53</v>
+      </c>
+      <c r="S11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>14</v>
       </c>
@@ -697,7 +859,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>18</v>
       </c>
@@ -729,7 +891,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>17</v>
       </c>
@@ -991,9 +1153,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="B23:K23"/>
     <mergeCell ref="B1:K1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>